<commit_message>
feat: add Stratified Cross-Validation and model complexity/size heuristics to all notebooks
</commit_message>
<xml_diff>
--- a/fact_abastecimiento_logistica/outputs/02_configuracion_modelo.xlsx
+++ b/fact_abastecimiento_logistica/outputs/02_configuracion_modelo.xlsx
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Capa 1: 64 Neuronas, Capa 2: 32 Neuronas</t>
+          <t>Capa 1: 32 Neuronas, Capa 2: 20 Neuronas</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>75.70440000000001</v>
+        <v>75.7278</v>
       </c>
     </row>
     <row r="11">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>78.2503</v>
+        <v>77.8708</v>
       </c>
     </row>
     <row r="12">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>77.15949999999999</v>
+        <v>77.3152</v>
       </c>
     </row>
     <row r="13">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.468916</v>
+        <v>0.480469</v>
       </c>
     </row>
     <row r="14">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.483028</v>
+        <v>0.49476</v>
       </c>
     </row>
   </sheetData>

</xml_diff>